<commit_message>
pillers 3 encapsulation learn about and make getters and setters
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4C20E4-26DC-4645-B5E5-38705AC4F1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6887843-7AF8-4177-9E11-3885CDE2F341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
   <si>
     <t>video</t>
   </si>
@@ -184,6 +184,52 @@
   </si>
   <si>
     <t>https://youtu.be/UrmbrygUyzU</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day13</t>
+  </si>
+  <si>
+    <t>Day14</t>
+  </si>
+  <si>
+    <t>Day15</t>
+  </si>
+  <si>
+    <t>Day16</t>
+  </si>
+  <si>
+    <t>Day17</t>
+  </si>
+  <si>
+    <t>https://youtu.be/GsqLYUAYGO4</t>
+  </si>
+  <si>
+    <t>oops piller2- polymorphism ,run time polymorphism(method overriding), compile time polymorphism(method overloading)</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>oops piller3-encapsulation ,packages</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>extra</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>how java programming language introduce ,why java compile and intreprate language and jvm jre and jdk</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/LBqE4YOvhyc</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/pdS8_smlsXA</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-VOO76LOCv4</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -727,7 +773,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F72"/>
+  <dimension ref="B1:F73"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -788,194 +834,220 @@
     </row>
     <row r="6" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="4" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="6"/>
       <c r="F6" s="6"/>
     </row>
     <row r="7" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B7" s="4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B8" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="6"/>
+        <v>59</v>
+      </c>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-    </row>
-    <row r="10" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="4" t="s">
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+    </row>
+    <row r="11" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="10"/>
-    </row>
-    <row r="11" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>28</v>
-      </c>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D13" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-    </row>
-    <row r="13" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B13" s="4" t="s">
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+    </row>
+    <row r="14" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
     <row r="16" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B17" s="4"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
+    <row r="17" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>47</v>
+      </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="4"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B19" s="4"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="6"/>
+    <row r="19" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B20" s="4"/>
+    <row r="20" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="4" t="s">
+        <v>50</v>
+      </c>
       <c r="C20" s="5"/>
       <c r="D20" s="6"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="4"/>
+      <c r="B21" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="C21" s="5"/>
       <c r="D21" s="6"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B22" s="4"/>
+      <c r="B22" s="4" t="s">
+        <v>52</v>
+      </c>
       <c r="C22" s="5"/>
       <c r="D22" s="6"/>
       <c r="E22" s="5"/>
@@ -1002,7 +1074,13 @@
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
     </row>
-    <row r="26" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" s="4"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+    </row>
     <row r="27" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="29" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1032,39 +1110,43 @@
     <row r="53" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="54" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="55" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="58" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="59" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="60" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="61" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="62" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="7"/>
-    </row>
-    <row r="64" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="7"/>
+    </row>
+    <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="68" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="69" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="70" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="71" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>
-    <hyperlink ref="D10" r:id="rId1" xr:uid="{DF269509-726B-4C5C-9333-9446C5C21ECE}"/>
-    <hyperlink ref="D11" r:id="rId2" xr:uid="{FF7E07CF-23E0-47CD-B6D1-B1A4E392A378}"/>
-    <hyperlink ref="E10" r:id="rId3" xr:uid="{8E9EC36F-3F87-451C-A752-2521C593A2BC}"/>
-    <hyperlink ref="E11" r:id="rId4" xr:uid="{4662B24C-6362-4A05-B0C4-E96F39915972}"/>
-    <hyperlink ref="F11" r:id="rId5" xr:uid="{8A344E58-E167-420E-9C96-8E11789B88BD}"/>
-    <hyperlink ref="D12" r:id="rId6" xr:uid="{45ACF002-962E-41BF-92DC-1CA7653639E8}"/>
-    <hyperlink ref="D14" r:id="rId7" xr:uid="{9FD94FC2-C602-4E71-AD25-2975A6ECDC53}"/>
-    <hyperlink ref="D15" r:id="rId8" xr:uid="{959E257A-0147-4C90-97D9-5042C0D6C251}"/>
-    <hyperlink ref="E8" r:id="rId9" xr:uid="{649FA6F5-AE0A-40F0-B9B0-3F91F8534DAE}"/>
-    <hyperlink ref="D9" r:id="rId10" xr:uid="{F1FD8ACC-B4B3-44C1-B1FA-B2E92E167D3C}"/>
-    <hyperlink ref="D16" r:id="rId11" xr:uid="{47F67C17-75C3-47D0-BCE3-0D20E3D624D0}"/>
+    <hyperlink ref="D11" r:id="rId1" xr:uid="{DF269509-726B-4C5C-9333-9446C5C21ECE}"/>
+    <hyperlink ref="D12" r:id="rId2" xr:uid="{FF7E07CF-23E0-47CD-B6D1-B1A4E392A378}"/>
+    <hyperlink ref="E11" r:id="rId3" xr:uid="{8E9EC36F-3F87-451C-A752-2521C593A2BC}"/>
+    <hyperlink ref="E12" r:id="rId4" xr:uid="{4662B24C-6362-4A05-B0C4-E96F39915972}"/>
+    <hyperlink ref="F12" r:id="rId5" xr:uid="{8A344E58-E167-420E-9C96-8E11789B88BD}"/>
+    <hyperlink ref="D13" r:id="rId6" xr:uid="{45ACF002-962E-41BF-92DC-1CA7653639E8}"/>
+    <hyperlink ref="D15" r:id="rId7" xr:uid="{9FD94FC2-C602-4E71-AD25-2975A6ECDC53}"/>
+    <hyperlink ref="D16" r:id="rId8" xr:uid="{959E257A-0147-4C90-97D9-5042C0D6C251}"/>
+    <hyperlink ref="E9" r:id="rId9" xr:uid="{649FA6F5-AE0A-40F0-B9B0-3F91F8534DAE}"/>
+    <hyperlink ref="D10" r:id="rId10" xr:uid="{F1FD8ACC-B4B3-44C1-B1FA-B2E92E167D3C}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{47F67C17-75C3-47D0-BCE3-0D20E3D624D0}"/>
+    <hyperlink ref="D6" r:id="rId12" xr:uid="{EC6C7C3C-328E-4907-BCCE-7CD554A870BF}"/>
+    <hyperlink ref="E8" r:id="rId13" xr:uid="{A0F3E2B6-4627-4358-90DD-1EE14B81FE62}"/>
+    <hyperlink ref="D19" r:id="rId14" xr:uid="{69BD34D7-C27B-40C9-96A9-76313FBE3C79}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
repete video encapsulation learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6887843-7AF8-4177-9E11-3885CDE2F341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44BA9A8-E102-4DD8-8A1D-5596E11C46CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -209,10 +209,6 @@
     <phoneticPr fontId="5"/>
   </si>
   <si>
-    <t>oops piller3-encapsulation ,packages</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
     <t>extra</t>
     <phoneticPr fontId="5"/>
   </si>
@@ -230,6 +226,10 @@
   </si>
   <si>
     <t>https://youtu.be/-VOO76LOCv4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>oops piller3-encapsulation ,packages and why make getters and setters  to access data</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -834,13 +834,13 @@
     </row>
     <row r="6" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>58</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -871,7 +871,7 @@
         <v>15</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F8" s="5"/>
     </row>
@@ -1018,10 +1018,10 @@
         <v>49</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>

</xml_diff>

<commit_message>
piller 4 abstract class and interface be leaned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44BA9A8-E102-4DD8-8A1D-5596E11C46CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565008F3-4689-49BF-8E71-A496F91B3213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
   <si>
     <t>video</t>
   </si>
@@ -231,13 +231,20 @@
   <si>
     <t>oops piller3-encapsulation ,packages and why make getters and setters  to access data</t>
     <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>oops pillers4 abstraction and piller 1 polymorphism repeate</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-L9BcU6Xk2c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -288,6 +295,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -426,7 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -466,6 +479,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -778,10 +797,10 @@
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="117" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.453125" customWidth="1"/>
+    <col min="3" max="3" width="126.54296875" customWidth="1"/>
+    <col min="4" max="4" width="47.7265625" customWidth="1"/>
+    <col min="5" max="5" width="39.90625" customWidth="1"/>
+    <col min="6" max="6" width="33.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -818,10 +837,10 @@
       </c>
     </row>
     <row r="5" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="14" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="6" t="s">
@@ -833,10 +852,10 @@
       <c r="F5" s="6"/>
     </row>
     <row r="6" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="14" t="s">
         <v>56</v>
       </c>
       <c r="D6" s="8" t="s">
@@ -846,10 +865,10 @@
       <c r="F6" s="6"/>
     </row>
     <row r="7" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -861,10 +880,10 @@
       <c r="F7" s="6"/>
     </row>
     <row r="8" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="6" t="s">
@@ -876,10 +895,10 @@
       <c r="F8" s="5"/>
     </row>
     <row r="9" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="14" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -891,10 +910,10 @@
       <c r="F9" s="6"/>
     </row>
     <row r="10" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="14" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="8" t="s">
@@ -903,11 +922,11 @@
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="4" t="s">
+    <row r="11" spans="2:6" ht="22" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B11" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="14" t="s">
         <v>22</v>
       </c>
       <c r="D11" s="8" t="s">
@@ -918,11 +937,11 @@
       </c>
       <c r="F11" s="10"/>
     </row>
-    <row r="12" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="4" t="s">
+    <row r="12" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B12" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="14" t="s">
         <v>26</v>
       </c>
       <c r="D12" s="9" t="s">
@@ -935,11 +954,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="4" t="s">
+    <row r="13" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="14" t="s">
         <v>31</v>
       </c>
       <c r="D13" s="8" t="s">
@@ -949,10 +968,10 @@
       <c r="F13" s="11"/>
     </row>
     <row r="14" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="14" t="s">
         <v>33</v>
       </c>
       <c r="D14" s="6" t="s">
@@ -961,11 +980,11 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="4" t="s">
+    <row r="15" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B15" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="14" t="s">
         <v>34</v>
       </c>
       <c r="D15" s="8" t="s">
@@ -974,11 +993,11 @@
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="4" t="s">
+    <row r="16" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B16" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="14" t="s">
         <v>36</v>
       </c>
       <c r="D16" s="8" t="s">
@@ -987,11 +1006,11 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="4" t="s">
+    <row r="17" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B17" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D17" s="8" t="s">
@@ -1001,10 +1020,10 @@
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="14" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -1013,11 +1032,11 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="4" t="s">
+    <row r="19" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B19" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="14" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="8" t="s">
@@ -1027,16 +1046,20 @@
       <c r="F19" s="5"/>
     </row>
     <row r="20" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
+      <c r="C20" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
     <row r="21" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="15" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="5"/>
@@ -1045,7 +1068,7 @@
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C22" s="5"/>

</xml_diff>

<commit_message>
AutoBoxing, Abstract classes & POJOs | Why only one public class in java file be learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40087AB6-B7D0-449F-9349-495C2789B2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2FC28F-841E-4470-9C0F-E4EF9D7A9BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>video</t>
   </si>
@@ -283,6 +283,14 @@
   </si>
   <si>
     <t>https://youtu.be/YLLFHuStkW8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/crVwHNW-fX8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">AutoBoxing, Abstract classes &amp; POJOs | Why only one public class in java file </t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1140,12 +1148,16 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B24" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="5"/>
+      <c r="C24" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>76</v>
+      </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
@@ -1299,6 +1311,7 @@
     <hyperlink ref="D21" r:id="rId16" xr:uid="{3A7EB145-EB16-4588-9378-0D91EDD6D780}"/>
     <hyperlink ref="D20" r:id="rId17" xr:uid="{2856E729-1015-44E4-B221-4D417D6A63E8}"/>
     <hyperlink ref="D23" r:id="rId18" xr:uid="{367C972B-3961-459D-8845-0E3A060B8C8D}"/>
+    <hyperlink ref="D24" r:id="rId19" xr:uid="{4B843059-7ECA-4527-AFF5-4C5BA73E740E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day20 java nested classes type learned like static method inner method etc
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2FC28F-841E-4470-9C0F-E4EF9D7A9BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D23502-7AAC-4558-9614-2925CE8DDBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="80">
   <si>
     <t>video</t>
   </si>
@@ -291,6 +291,14 @@
   </si>
   <si>
     <t xml:space="preserve">AutoBoxing, Abstract classes &amp; POJOs | Why only one public class in java file </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/0LaBK28_470</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Nested Classes type| 1)Static Nested, 2)Inner, 3)Local &amp;4)Anonymous Classes</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1161,12 +1169,16 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B25" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="5"/>
+      <c r="C25" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>78</v>
+      </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
@@ -1312,6 +1324,7 @@
     <hyperlink ref="D20" r:id="rId17" xr:uid="{2856E729-1015-44E4-B221-4D417D6A63E8}"/>
     <hyperlink ref="D23" r:id="rId18" xr:uid="{367C972B-3961-459D-8845-0E3A060B8C8D}"/>
     <hyperlink ref="D24" r:id="rId19" xr:uid="{4B843059-7ECA-4527-AFF5-4C5BA73E740E}"/>
+    <hyperlink ref="D25" r:id="rId20" xr:uid="{DE3D6C26-B1C0-42E9-B87B-EC8B1F45C4CB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Immutable Classes in Java | How to Create Immutable Objects  and its rule
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D23502-7AAC-4558-9614-2925CE8DDBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34BC13E-F4DE-498E-9937-159151417170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
   <si>
     <t>video</t>
   </si>
@@ -299,6 +299,14 @@
   </si>
   <si>
     <t>Java Nested Classes type| 1)Static Nested, 2)Inner, 3)Local &amp;4)Anonymous Classes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">learn Immutable Classes in Java | How to Create Immutable Objects </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/vgQVz5OdFws</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1182,12 +1190,16 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B26" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="5"/>
+      <c r="C26" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>81</v>
+      </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
@@ -1325,6 +1337,7 @@
     <hyperlink ref="D23" r:id="rId18" xr:uid="{367C972B-3961-459D-8845-0E3A060B8C8D}"/>
     <hyperlink ref="D24" r:id="rId19" xr:uid="{4B843059-7ECA-4527-AFF5-4C5BA73E740E}"/>
     <hyperlink ref="D25" r:id="rId20" xr:uid="{DE3D6C26-B1C0-42E9-B87B-EC8B1F45C4CB}"/>
+    <hyperlink ref="D26" r:id="rId21" xr:uid="{0D70FCBF-C928-4B39-8C62-F06B7AB9AD07}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Object Class in java and its corebehavour==> core biheviours(equals, hashCode, toString,getclass)
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34BC13E-F4DE-498E-9937-159151417170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962A2B43-1E06-44A3-9EA6-61FFBCD82B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="92">
   <si>
     <t>video</t>
   </si>
@@ -307,6 +307,38 @@
   </si>
   <si>
     <t>https://youtu.be/vgQVz5OdFws</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/541Zpv6sOKo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day25</t>
+  </si>
+  <si>
+    <t>Day26</t>
+  </si>
+  <si>
+    <t>Day27</t>
+  </si>
+  <si>
+    <t>Day28</t>
+  </si>
+  <si>
+    <t>Day29</t>
+  </si>
+  <si>
+    <t>Day30</t>
+  </si>
+  <si>
+    <t>Day31</t>
+  </si>
+  <si>
+    <t>Day32</t>
+  </si>
+  <si>
+    <t>learn Object Class (equals, hashCode, toString)  which is most important in java</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -859,7 +891,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F81"/>
+  <dimension ref="B1:F91"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -1203,12 +1235,16 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B27" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="5"/>
+      <c r="C27" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>82</v>
+      </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
@@ -1230,51 +1266,127 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B30" s="14"/>
-      <c r="C30" s="4"/>
+    <row r="30" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B30" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="13"/>
       <c r="D30" s="5"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B31" s="14"/>
-      <c r="C31" s="4"/>
+    <row r="31" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="13"/>
       <c r="D31" s="5"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B32" s="14"/>
-      <c r="C32" s="4"/>
+    <row r="32" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B32" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" s="13"/>
       <c r="D32" s="5"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B33" s="14"/>
-      <c r="C33" s="4"/>
+    <row r="33" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B33" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="13"/>
       <c r="D33" s="5"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B34" s="14"/>
-      <c r="C34" s="4"/>
+    <row r="34" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B34" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" s="13"/>
       <c r="D34" s="5"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
-    <row r="35" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B35" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B36" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" s="13"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B37" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" s="13"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+    </row>
+    <row r="38" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B38" s="14"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+    </row>
+    <row r="39" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B39" s="14"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+    </row>
+    <row r="40" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B40" s="14"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+    </row>
+    <row r="41" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B41" s="14"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+    </row>
+    <row r="42" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B42" s="14"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+    </row>
+    <row r="43" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B43" s="14"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+    </row>
+    <row r="44" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B44" s="14"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+    </row>
     <row r="45" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="47" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1295,25 +1407,35 @@
     <row r="62" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="64" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B72" s="6"/>
-    </row>
-    <row r="73" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="68" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="71" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B82" s="6"/>
+    </row>
+    <row r="83" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>
@@ -1338,6 +1460,7 @@
     <hyperlink ref="D24" r:id="rId19" xr:uid="{4B843059-7ECA-4527-AFF5-4C5BA73E740E}"/>
     <hyperlink ref="D25" r:id="rId20" xr:uid="{DE3D6C26-B1C0-42E9-B87B-EC8B1F45C4CB}"/>
     <hyperlink ref="D26" r:id="rId21" xr:uid="{0D70FCBF-C928-4B39-8C62-F06B7AB9AD07}"/>
+    <hyperlink ref="D27" r:id="rId22" xr:uid="{310D84FF-6DA2-463A-84E6-CFDFC7A05731}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java input output Deep Dive | InputStreams, System.in, Scanner vs BufferedReader
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF5D66B-4B12-4061-BDFE-6B634FD0261A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D478389-5FDA-455F-8673-B79BB74D2A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="96">
   <si>
     <t>video</t>
   </si>
@@ -343,6 +343,18 @@
   </si>
   <si>
     <t xml:space="preserve">Java Enums | Why Not Use int/String for Constants? </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/oXhy5dT-0Qs</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/yfMWLZGEPwo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java I/O Deep Dive | InputStreams, System.in, Scanner vs BufferedReader</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1252,23 +1264,29 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B28" s="14" t="s">
         <v>72</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D28" s="5"/>
+      <c r="D28" s="7" t="s">
+        <v>93</v>
+      </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B29" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="5"/>
+      <c r="C29" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>94</v>
+      </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
@@ -1467,6 +1485,8 @@
     <hyperlink ref="D25" r:id="rId20" xr:uid="{DE3D6C26-B1C0-42E9-B87B-EC8B1F45C4CB}"/>
     <hyperlink ref="D26" r:id="rId21" xr:uid="{0D70FCBF-C928-4B39-8C62-F06B7AB9AD07}"/>
     <hyperlink ref="D27" r:id="rId22" xr:uid="{310D84FF-6DA2-463A-84E6-CFDFC7A05731}"/>
+    <hyperlink ref="D28" r:id="rId23" xr:uid="{F10E4049-1CEF-4D6E-9B57-20A1721206AA}"/>
+    <hyperlink ref="D29" r:id="rId24" xr:uid="{C9C8A820-1D7D-4471-A6BC-D4955334C600}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
learn about Java Strings | String Pool, Immutability, Internals part of string ets
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D478389-5FDA-455F-8673-B79BB74D2A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D65F2D-90B2-4A78-A26A-71999741D74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="98">
   <si>
     <t>video</t>
   </si>
@@ -355,6 +355,14 @@
   </si>
   <si>
     <t>Java I/O Deep Dive | InputStreams, System.in, Scanner vs BufferedReader</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Strings | String Pool, Immutability, Internals</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/N0b8lRXtK_Y</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1290,12 +1298,16 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B30" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="5"/>
+      <c r="C30" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>97</v>
+      </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
@@ -1487,6 +1499,7 @@
     <hyperlink ref="D27" r:id="rId22" xr:uid="{310D84FF-6DA2-463A-84E6-CFDFC7A05731}"/>
     <hyperlink ref="D28" r:id="rId23" xr:uid="{F10E4049-1CEF-4D6E-9B57-20A1721206AA}"/>
     <hyperlink ref="D29" r:id="rId24" xr:uid="{C9C8A820-1D7D-4471-A6BC-D4955334C600}"/>
+    <hyperlink ref="D30" r:id="rId25" xr:uid="{86E03E88-ED36-45CE-BD93-8D8A4AC6E3FA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
learn String method and stringbuilder and stringbuffer methods
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D65F2D-90B2-4A78-A26A-71999741D74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC63FB74-E0A3-4C81-94EF-026BC346FD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="100">
   <si>
     <t>video</t>
   </si>
@@ -363,6 +363,14 @@
   </si>
   <si>
     <t>https://youtu.be/N0b8lRXtK_Y</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/JcAD9a22Rks</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Strings Part 2 | All String Methods + StringBuilder vs StringBuffer</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1311,12 +1319,16 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B31" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="5"/>
+      <c r="C31" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>98</v>
+      </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
@@ -1500,6 +1512,7 @@
     <hyperlink ref="D28" r:id="rId23" xr:uid="{F10E4049-1CEF-4D6E-9B57-20A1721206AA}"/>
     <hyperlink ref="D29" r:id="rId24" xr:uid="{C9C8A820-1D7D-4471-A6BC-D4955334C600}"/>
     <hyperlink ref="D30" r:id="rId25" xr:uid="{86E03E88-ED36-45CE-BD93-8D8A4AC6E3FA}"/>
+    <hyperlink ref="D31" r:id="rId26" xr:uid="{89254919-8F85-4394-AF57-F0B845E77456}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
learn about Generic and opcasting and downcasting
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC63FB74-E0A3-4C81-94EF-026BC346FD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958CBF29-5F23-4E39-812C-8D11D7F67276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
   <si>
     <t>video</t>
   </si>
@@ -371,6 +371,14 @@
   </si>
   <si>
     <t>Java Strings Part 2 | All String Methods + StringBuilder vs StringBuffer</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Y7X_ReDF3x8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java Generics Deep Dive | Bounded Types using extends </t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1332,12 +1340,16 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B32" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="5"/>
+      <c r="C32" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>100</v>
+      </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
@@ -1513,6 +1525,7 @@
     <hyperlink ref="D29" r:id="rId24" xr:uid="{C9C8A820-1D7D-4471-A6BC-D4955334C600}"/>
     <hyperlink ref="D30" r:id="rId25" xr:uid="{86E03E88-ED36-45CE-BD93-8D8A4AC6E3FA}"/>
     <hyperlink ref="D31" r:id="rId26" xr:uid="{89254919-8F85-4394-AF57-F0B845E77456}"/>
+    <hyperlink ref="D32" r:id="rId27" xr:uid="{AFAA2CD6-D3A0-4881-B45F-82D2F742DAB6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
wildcards in generic learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958CBF29-5F23-4E39-812C-8D11D7F67276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63B77FE-1C50-4EC7-9C92-8B0D68BF89AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="104">
   <si>
     <t>video</t>
   </si>
@@ -379,6 +379,14 @@
   </si>
   <si>
     <t xml:space="preserve">Java Generics Deep Dive | Bounded Types using extends </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Wildcards in Generics |  extends, ? super | Java Full Course #28</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Opb2q2WSyes</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1353,12 +1361,16 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B33" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="5"/>
+      <c r="C33" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>103</v>
+      </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
@@ -1526,6 +1538,7 @@
     <hyperlink ref="D30" r:id="rId25" xr:uid="{86E03E88-ED36-45CE-BD93-8D8A4AC6E3FA}"/>
     <hyperlink ref="D31" r:id="rId26" xr:uid="{89254919-8F85-4394-AF57-F0B845E77456}"/>
     <hyperlink ref="D32" r:id="rId27" xr:uid="{AFAA2CD6-D3A0-4881-B45F-82D2F742DAB6}"/>
+    <hyperlink ref="D33" r:id="rId28" xr:uid="{CBCF07B4-DB1D-473C-BC1B-880C22740F2E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
only therory learned about Java Collection Framework Explained | Data Structures + Complete
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63B77FE-1C50-4EC7-9C92-8B0D68BF89AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F0313C-FAC0-4E19-BC07-A5641F6EBFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="106">
   <si>
     <t>video</t>
   </si>
@@ -387,6 +387,14 @@
   </si>
   <si>
     <t>https://youtu.be/Opb2q2WSyes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/mW2OO6d6_BE</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">theory only-Java Collection Framework Explained | Data Structures + Complete Hierarchy </t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1374,12 +1382,16 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B34" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="5"/>
+      <c r="C34" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>104</v>
+      </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
@@ -1539,6 +1551,7 @@
     <hyperlink ref="D31" r:id="rId26" xr:uid="{89254919-8F85-4394-AF57-F0B845E77456}"/>
     <hyperlink ref="D32" r:id="rId27" xr:uid="{AFAA2CD6-D3A0-4881-B45F-82D2F742DAB6}"/>
     <hyperlink ref="D33" r:id="rId28" xr:uid="{CBCF07B4-DB1D-473C-BC1B-880C22740F2E}"/>
+    <hyperlink ref="D34" r:id="rId29" xr:uid="{E82E30AB-AC4C-42BD-B3D7-67815CEDAD92}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Iterable Interface in Java | Why Iterator Exists?
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F0313C-FAC0-4E19-BC07-A5641F6EBFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C5AB8-B8E6-4A6B-83AD-36F178144ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="108">
   <si>
     <t>video</t>
   </si>
@@ -395,6 +395,13 @@
   </si>
   <si>
     <t xml:space="preserve">theory only-Java Collection Framework Explained | Data Structures + Complete Hierarchy </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/LVwpxEZ6uMQ</t>
+  </si>
+  <si>
+    <t>Iterable Interface in Java | Why Iterator Exists?</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -947,7 +954,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F91"/>
+  <dimension ref="B1:F95"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -1399,8 +1406,12 @@
       <c r="B35" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="C35" s="13"/>
-      <c r="D35" s="5"/>
+      <c r="C35" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>106</v>
+      </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
@@ -1471,10 +1482,34 @@
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B45" s="14"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+    </row>
+    <row r="46" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B46" s="14"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B47" s="14"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+    </row>
+    <row r="48" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B48" s="14"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+    </row>
     <row r="49" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1501,25 +1536,29 @@
     <row r="72" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="73" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="74" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="76" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="77" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="81" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B82" s="6"/>
-    </row>
+    <row r="82" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="83" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="85" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B86" s="6"/>
+    </row>
     <row r="87" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="89" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="90" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Java Collection Interface Deep Dive | Methods & Internals  of that interface
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72C5AB8-B8E6-4A6B-83AD-36F178144ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958FE38B-F696-4A2F-B517-B8495F966A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="110">
   <si>
     <t>video</t>
   </si>
@@ -402,6 +402,14 @@
   </si>
   <si>
     <t>Iterable Interface in Java | Why Iterator Exists?</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Collection Interface Deep Dive | Methods &amp; Internals | Java Full Course #31</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/cazzzwdLAkQ</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1415,12 +1423,16 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B36" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="5"/>
+      <c r="C36" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>109</v>
+      </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
     </row>
@@ -1591,6 +1603,7 @@
     <hyperlink ref="D32" r:id="rId27" xr:uid="{AFAA2CD6-D3A0-4881-B45F-82D2F742DAB6}"/>
     <hyperlink ref="D33" r:id="rId28" xr:uid="{CBCF07B4-DB1D-473C-BC1B-880C22740F2E}"/>
     <hyperlink ref="D34" r:id="rId29" xr:uid="{E82E30AB-AC4C-42BD-B3D7-67815CEDAD92}"/>
+    <hyperlink ref="D36" r:id="rId30" xr:uid="{AE50B190-B349-4C86-8E57-E063E0ED48B4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Set & Map Interface in Java | Internal Working of HashMap, HashSet & TreeMap |
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958FE38B-F696-4A2F-B517-B8495F966A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C30415E-85C3-451C-9F43-448BCB780A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="124">
   <si>
     <t>video</t>
   </si>
@@ -410,6 +410,51 @@
   </si>
   <si>
     <t>https://youtu.be/cazzzwdLAkQ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/OfNtIOGDqzY</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java List Interface Deep Dive | ArrayList, LinkedList, Vector, Stack </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day33</t>
+  </si>
+  <si>
+    <t>Day34</t>
+  </si>
+  <si>
+    <t>Day35</t>
+  </si>
+  <si>
+    <t>Day36</t>
+  </si>
+  <si>
+    <t>Day37</t>
+  </si>
+  <si>
+    <t>Day38</t>
+  </si>
+  <si>
+    <t>Day39</t>
+  </si>
+  <si>
+    <t>Day40</t>
+  </si>
+  <si>
+    <t>Day41</t>
+  </si>
+  <si>
+    <t>Day42</t>
+  </si>
+  <si>
+    <t>https://youtu.be/kzZ1TlGTWmY</t>
+  </si>
+  <si>
+    <t>Set &amp; Map Interface in Java | Internal Working of HashMap, HashSet &amp; TreeMap</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1436,80 +1481,108 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B37" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="13"/>
-      <c r="D37" s="5"/>
+      <c r="C37" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>110</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B38" s="14"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="5"/>
+      <c r="B38" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>122</v>
+      </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
     <row r="39" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B39" s="14"/>
+      <c r="B39" s="14" t="s">
+        <v>113</v>
+      </c>
       <c r="C39" s="13"/>
       <c r="D39" s="5"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B40" s="14"/>
+      <c r="B40" s="14" t="s">
+        <v>114</v>
+      </c>
       <c r="C40" s="4"/>
       <c r="D40" s="5"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
     </row>
     <row r="41" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B41" s="14"/>
+      <c r="B41" s="14" t="s">
+        <v>115</v>
+      </c>
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B42" s="14"/>
+      <c r="B42" s="14" t="s">
+        <v>116</v>
+      </c>
       <c r="C42" s="4"/>
       <c r="D42" s="5"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
     </row>
     <row r="43" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B43" s="14"/>
+      <c r="B43" s="14" t="s">
+        <v>117</v>
+      </c>
       <c r="C43" s="4"/>
       <c r="D43" s="5"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
     </row>
     <row r="44" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B44" s="14"/>
+      <c r="B44" s="14" t="s">
+        <v>118</v>
+      </c>
       <c r="C44" s="4"/>
       <c r="D44" s="5"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
     <row r="45" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B45" s="14"/>
+      <c r="B45" s="14" t="s">
+        <v>119</v>
+      </c>
       <c r="C45" s="4"/>
       <c r="D45" s="5"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
     </row>
     <row r="46" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B46" s="14"/>
+      <c r="B46" s="14" t="s">
+        <v>120</v>
+      </c>
       <c r="C46" s="4"/>
       <c r="D46" s="5"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
     <row r="47" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B47" s="14"/>
+      <c r="B47" s="14" t="s">
+        <v>121</v>
+      </c>
       <c r="C47" s="4"/>
       <c r="D47" s="5"/>
       <c r="E47" s="4"/>
@@ -1604,6 +1677,7 @@
     <hyperlink ref="D33" r:id="rId28" xr:uid="{CBCF07B4-DB1D-473C-BC1B-880C22740F2E}"/>
     <hyperlink ref="D34" r:id="rId29" xr:uid="{E82E30AB-AC4C-42BD-B3D7-67815CEDAD92}"/>
     <hyperlink ref="D36" r:id="rId30" xr:uid="{AE50B190-B349-4C86-8E57-E063E0ED48B4}"/>
+    <hyperlink ref="D37" r:id="rId31" xr:uid="{FEF26AD1-9A6F-45F7-A679-B522519A40A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Set & Map Methods Explained | EnumMaps, IdentityHashMaps & More
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C30415E-85C3-451C-9F43-448BCB780A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A27780-A088-4359-B34D-D23DF086DC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="126">
   <si>
     <t>video</t>
   </si>
@@ -455,6 +455,14 @@
   </si>
   <si>
     <t>Set &amp; Map Interface in Java | Internal Working of HashMap, HashSet &amp; TreeMap</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Set &amp; Map Methods Explained | EnumMaps, IdentityHashMaps &amp; More in collection framework</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/b1Uj_2MPBwA</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1507,12 +1515,16 @@
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B39" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="C39" s="13"/>
-      <c r="D39" s="5"/>
+      <c r="C39" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>125</v>
+      </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
@@ -1678,6 +1690,7 @@
     <hyperlink ref="D34" r:id="rId29" xr:uid="{E82E30AB-AC4C-42BD-B3D7-67815CEDAD92}"/>
     <hyperlink ref="D36" r:id="rId30" xr:uid="{AE50B190-B349-4C86-8E57-E063E0ED48B4}"/>
     <hyperlink ref="D37" r:id="rId31" xr:uid="{FEF26AD1-9A6F-45F7-A679-B522519A40A0}"/>
+    <hyperlink ref="D39" r:id="rId32" xr:uid="{7226FF78-BB1C-4916-8EFC-786E81556C1D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java Lambdas & Functional Interfaces | Comparator Interface  learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A27780-A088-4359-B34D-D23DF086DC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7406AAA0-56F8-4C73-B5A0-FF05EF25BFB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="139">
   <si>
     <t>video</t>
   </si>
@@ -464,6 +464,50 @@
   <si>
     <t>https://youtu.be/b1Uj_2MPBwA</t>
     <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/zj0-JIc5oPw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Queue Interface Deep Dive | PriorityQueue &amp; Heap Explained | Java Full Course #35</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day43</t>
+  </si>
+  <si>
+    <t>Day44</t>
+  </si>
+  <si>
+    <t>Day45</t>
+  </si>
+  <si>
+    <t>Day46</t>
+  </si>
+  <si>
+    <t>Day47</t>
+  </si>
+  <si>
+    <t>Day48</t>
+  </si>
+  <si>
+    <t>Day49</t>
+  </si>
+  <si>
+    <t>https://youtu.be/uUo7AV02vJM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Comparable Interface in Java | Collections class | Comparing Objects | Java Full Course #36</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Lambdas &amp; Functional Interfaces | Comparator Interface | Java Full Course #37</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/0V-w2BywAM0</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1059,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F95"/>
+  <dimension ref="B1:F102"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -1528,21 +1572,29 @@
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B40" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="5"/>
+      <c r="C40" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>126</v>
+      </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B41" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="C41" s="4"/>
-      <c r="D41" s="5"/>
+      <c r="C41" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>135</v>
+      </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
@@ -1550,8 +1602,12 @@
       <c r="B42" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C42" s="4"/>
-      <c r="D42" s="5"/>
+      <c r="C42" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
     </row>
@@ -1559,7 +1615,7 @@
       <c r="B43" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C43" s="4"/>
+      <c r="C43" s="13"/>
       <c r="D43" s="5"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
@@ -1568,7 +1624,7 @@
       <c r="B44" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="C44" s="4"/>
+      <c r="C44" s="13"/>
       <c r="D44" s="5"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
@@ -1577,7 +1633,7 @@
       <c r="B45" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="C45" s="4"/>
+      <c r="C45" s="13"/>
       <c r="D45" s="5"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
@@ -1586,7 +1642,7 @@
       <c r="B46" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C46" s="4"/>
+      <c r="C46" s="13"/>
       <c r="D46" s="5"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
@@ -1595,34 +1651,90 @@
       <c r="B47" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="4"/>
+      <c r="C47" s="13"/>
       <c r="D47" s="5"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B48" s="14"/>
-      <c r="C48" s="4"/>
+      <c r="B48" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C48" s="13"/>
       <c r="D48" s="5"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="50" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="51" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="52" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="53" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B49" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C49" s="13"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+    </row>
+    <row r="50" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B50" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C50" s="13"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B51" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" s="13"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+    </row>
+    <row r="52" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B52" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C52" s="13"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+    </row>
+    <row r="53" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B53" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="C53" s="13"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+    </row>
+    <row r="54" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B54" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C54" s="13"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+    </row>
+    <row r="55" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B55" s="14"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+    </row>
+    <row r="56" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="58" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="59" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1637,25 +1749,32 @@
     <row r="76" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="77" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="81" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="82" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="83" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="84" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="85" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B86" s="6"/>
-    </row>
+    <row r="86" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="87" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="89" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="90" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="91" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="92" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B93" s="6"/>
+    </row>
     <row r="94" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="97" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="98" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="100" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="101" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="102" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>
@@ -1691,6 +1810,8 @@
     <hyperlink ref="D36" r:id="rId30" xr:uid="{AE50B190-B349-4C86-8E57-E063E0ED48B4}"/>
     <hyperlink ref="D37" r:id="rId31" xr:uid="{FEF26AD1-9A6F-45F7-A679-B522519A40A0}"/>
     <hyperlink ref="D39" r:id="rId32" xr:uid="{7226FF78-BB1C-4916-8EFC-786E81556C1D}"/>
+    <hyperlink ref="D40" r:id="rId33" xr:uid="{78A9599A-AEF5-4F06-8DA5-8117B1A48D54}"/>
+    <hyperlink ref="D41" r:id="rId34" xr:uid="{99C33FBE-1013-4477-8454-D61407138AC8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Lambdas & Functional Interface Deep Dive
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7406AAA0-56F8-4C73-B5A0-FF05EF25BFB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BF430B-8221-496B-8D0D-F94B3A0FD640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="141">
   <si>
     <t>video</t>
   </si>
@@ -508,6 +508,14 @@
   </si>
   <si>
     <t>https://youtu.be/0V-w2BywAM0</t>
+  </si>
+  <si>
+    <t>Lambdas &amp; Functional Interface Deep Dive | Method References &amp; Composition | Java Full Course #38</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/IsC0Ms2iFi8</t>
+    <phoneticPr fontId="5"/>
   </si>
 </sst>
 </file>
@@ -1611,12 +1619,16 @@
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B43" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C43" s="13"/>
-      <c r="D43" s="5"/>
+      <c r="C43" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>140</v>
+      </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
     </row>
@@ -1812,6 +1824,7 @@
     <hyperlink ref="D39" r:id="rId32" xr:uid="{7226FF78-BB1C-4916-8EFC-786E81556C1D}"/>
     <hyperlink ref="D40" r:id="rId33" xr:uid="{78A9599A-AEF5-4F06-8DA5-8117B1A48D54}"/>
     <hyperlink ref="D41" r:id="rId34" xr:uid="{99C33FBE-1013-4477-8454-D61407138AC8}"/>
+    <hyperlink ref="D43" r:id="rId35" xr:uid="{E93555C8-FD1E-4D79-937C-EEC2D85BC784}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Introduction to Java Streams | Creation & Architecture
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BF430B-8221-496B-8D0D-F94B3A0FD640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F1507A-2F84-43B3-A77C-37958EC3D711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="143">
   <si>
     <t>video</t>
   </si>
@@ -515,6 +515,14 @@
   </si>
   <si>
     <t>https://youtu.be/IsC0Ms2iFi8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-jHyDEXHr_U</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Java Streams | Creation &amp; Architecture </t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1632,12 +1640,16 @@
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
     </row>
-    <row r="44" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B44" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="C44" s="13"/>
-      <c r="D44" s="5"/>
+      <c r="C44" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>141</v>
+      </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
@@ -1825,6 +1837,7 @@
     <hyperlink ref="D40" r:id="rId33" xr:uid="{78A9599A-AEF5-4F06-8DA5-8117B1A48D54}"/>
     <hyperlink ref="D41" r:id="rId34" xr:uid="{99C33FBE-1013-4477-8454-D61407138AC8}"/>
     <hyperlink ref="D43" r:id="rId35" xr:uid="{E93555C8-FD1E-4D79-937C-EEC2D85BC784}"/>
+    <hyperlink ref="D44" r:id="rId36" xr:uid="{C2026BE5-1ED2-411B-9CCA-86537B50FDF2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java Stream Methods Deep Dive | All Intermediate & Terminal Operations |
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F1507A-2F84-43B3-A77C-37958EC3D711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6EB1F7-E2B1-44BC-9557-F679E94AC427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="155">
   <si>
     <t>video</t>
   </si>
@@ -523,6 +523,44 @@
   </si>
   <si>
     <t xml:space="preserve">Introduction to Java Streams | Creation &amp; Architecture </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day50</t>
+  </si>
+  <si>
+    <t>Day51</t>
+  </si>
+  <si>
+    <t>Day52</t>
+  </si>
+  <si>
+    <t>Day53</t>
+  </si>
+  <si>
+    <t>Day54</t>
+  </si>
+  <si>
+    <t>Day55</t>
+  </si>
+  <si>
+    <t>Day56</t>
+  </si>
+  <si>
+    <t>Day57</t>
+  </si>
+  <si>
+    <t>Day58</t>
+  </si>
+  <si>
+    <t>Day59</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xqfOH5EA8xo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java Stream Methods Deep Dive | All Intermediate &amp; Terminal Operations </t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1075,7 +1113,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F102"/>
+  <dimension ref="B1:F111"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -1653,12 +1691,16 @@
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B45" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="C45" s="13"/>
-      <c r="D45" s="5"/>
+      <c r="C45" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>153</v>
+      </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
     </row>
@@ -1744,21 +1786,95 @@
       <c r="F54" s="4"/>
     </row>
     <row r="55" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B55" s="14"/>
-      <c r="C55" s="4"/>
+      <c r="B55" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C55" s="13"/>
       <c r="D55" s="5"/>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
     </row>
-    <row r="56" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B56" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C56" s="13"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+    </row>
+    <row r="57" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B57" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="C57" s="13"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+    </row>
+    <row r="58" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B58" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C58" s="13"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+    </row>
+    <row r="59" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B59" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C59" s="13"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+    </row>
+    <row r="60" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B60" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="C60" s="13"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+    </row>
+    <row r="61" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B61" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C61" s="13"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+    </row>
+    <row r="62" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B62" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C62" s="13"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+    </row>
+    <row r="63" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B63" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="C63" s="13"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+    </row>
+    <row r="64" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B64" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C64" s="4"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+    </row>
     <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1775,30 +1891,39 @@
     <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B93" s="6"/>
-    </row>
-    <row r="94" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="97" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="98" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="100" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="101" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="102" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B102" s="6"/>
+    </row>
+    <row r="103" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="105" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="106" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="107" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="108" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="109" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="110" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="111" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>
@@ -1838,6 +1963,7 @@
     <hyperlink ref="D41" r:id="rId34" xr:uid="{99C33FBE-1013-4477-8454-D61407138AC8}"/>
     <hyperlink ref="D43" r:id="rId35" xr:uid="{E93555C8-FD1E-4D79-937C-EEC2D85BC784}"/>
     <hyperlink ref="D44" r:id="rId36" xr:uid="{C2026BE5-1ED2-411B-9CCA-86537B50FDF2}"/>
+    <hyperlink ref="D45" r:id="rId37" xr:uid="{95537796-E406-44F9-9BC7-FDDCA94D8C4D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java Optional Explained from Scratch | All Methods + Streams Integration | be learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6EB1F7-E2B1-44BC-9557-F679E94AC427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60248ABE-F524-4A50-A6DD-4F25B3BFE6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="157">
   <si>
     <t>video</t>
   </si>
@@ -561,6 +561,14 @@
   </si>
   <si>
     <t xml:space="preserve">Java Stream Methods Deep Dive | All Intermediate &amp; Terminal Operations </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Q75kCaNa35Y</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Optional Explained from Scratch | All Methods + Streams Integration</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1704,12 +1712,16 @@
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B46" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C46" s="13"/>
-      <c r="D46" s="5"/>
+      <c r="C46" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>155</v>
+      </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
@@ -1964,6 +1976,7 @@
     <hyperlink ref="D43" r:id="rId35" xr:uid="{E93555C8-FD1E-4D79-937C-EEC2D85BC784}"/>
     <hyperlink ref="D44" r:id="rId36" xr:uid="{C2026BE5-1ED2-411B-9CCA-86537B50FDF2}"/>
     <hyperlink ref="D45" r:id="rId37" xr:uid="{95537796-E406-44F9-9BC7-FDDCA94D8C4D}"/>
+    <hyperlink ref="D46" r:id="rId38" xr:uid="{FFCBE106-7313-4C15-9467-E4D2D3728E59}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Parallel Streams in Java Explained | Primitive Optional Classes | Java Full
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60248ABE-F524-4A50-A6DD-4F25B3BFE6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EC4EFC-6E0E-4F0C-84AD-2E492329DEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="159">
   <si>
     <t>video</t>
   </si>
@@ -569,6 +569,14 @@
   </si>
   <si>
     <t>Java Optional Explained from Scratch | All Methods + Streams Integration</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Parallel Streams in Java Explained | Primitive Optional Classes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/zrtVQ1ev_0w</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1725,12 +1733,16 @@
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B47" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="C47" s="13"/>
-      <c r="D47" s="5"/>
+      <c r="C47" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>158</v>
+      </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
@@ -1977,6 +1989,7 @@
     <hyperlink ref="D44" r:id="rId36" xr:uid="{C2026BE5-1ED2-411B-9CCA-86537B50FDF2}"/>
     <hyperlink ref="D45" r:id="rId37" xr:uid="{95537796-E406-44F9-9BC7-FDDCA94D8C4D}"/>
     <hyperlink ref="D46" r:id="rId38" xr:uid="{FFCBE106-7313-4C15-9467-E4D2D3728E59}"/>
+    <hyperlink ref="D47" r:id="rId39" xr:uid="{9E9CFD17-8B4E-4159-A428-447A65AE33B9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java Exception Handling from Scratch | Exceptions vs Errors | be learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EC4EFC-6E0E-4F0C-84AD-2E492329DEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F9F13D-2F53-4D4C-B8DF-AEA5C4A884C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="161">
   <si>
     <t>video</t>
   </si>
@@ -577,6 +577,14 @@
   </si>
   <si>
     <t>https://youtu.be/zrtVQ1ev_0w</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Exception Handling from Scratch | Exceptions vs Errors |</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/mJg9iQZJEpw</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1746,12 +1754,16 @@
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
-    <row r="48" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B48" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="13"/>
-      <c r="D48" s="5"/>
+      <c r="C48" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>160</v>
+      </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
     </row>
@@ -1990,6 +2002,7 @@
     <hyperlink ref="D45" r:id="rId37" xr:uid="{95537796-E406-44F9-9BC7-FDDCA94D8C4D}"/>
     <hyperlink ref="D46" r:id="rId38" xr:uid="{FFCBE106-7313-4C15-9467-E4D2D3728E59}"/>
     <hyperlink ref="D47" r:id="rId39" xr:uid="{9E9CFD17-8B4E-4159-A428-447A65AE33B9}"/>
+    <hyperlink ref="D48" r:id="rId40" xr:uid="{EEFC57CB-B74A-4C45-8650-090249CDC424}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Exception Hierarchy Deep Dive | throw vs throws | Custom Exceptions
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F9F13D-2F53-4D4C-B8DF-AEA5C4A884C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49519F99-9DA3-4537-B939-6C8648A74387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="163">
   <si>
     <t>video</t>
   </si>
@@ -585,6 +585,14 @@
   </si>
   <si>
     <t>https://youtu.be/mJg9iQZJEpw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Exception Hierarchy Deep Dive | throw vs throws | Custom Exceptions | Java Full Course #44</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/xTxscoajikw</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1767,12 +1775,16 @@
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B49" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C49" s="13"/>
-      <c r="D49" s="5"/>
+      <c r="C49" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>162</v>
+      </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
     </row>
@@ -2003,6 +2015,7 @@
     <hyperlink ref="D46" r:id="rId38" xr:uid="{FFCBE106-7313-4C15-9467-E4D2D3728E59}"/>
     <hyperlink ref="D47" r:id="rId39" xr:uid="{9E9CFD17-8B4E-4159-A428-447A65AE33B9}"/>
     <hyperlink ref="D48" r:id="rId40" xr:uid="{EEFC57CB-B74A-4C45-8650-090249CDC424}"/>
+    <hyperlink ref="D49" r:id="rId41" xr:uid="{E4D9CAFF-0AF5-4837-B77F-00BD2850517C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Java Thread Creation & Lifecycle Explained be learned
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319AF2EA-2FAC-4FFA-9BC2-A244FC55D010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC946E34-9269-48D1-A717-45622408BF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="171">
   <si>
     <t>video</t>
   </si>
@@ -593,6 +593,38 @@
   </si>
   <si>
     <t>https://youtu.be/xTxscoajikw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Memory Management Explained in Depth | Stack, Heap, Method Area &amp; PC | Java Full Course #45</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/kjETbH63Pco</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Heap Memory Deep Dive | Garbage Collection Algorithms Explained | Java Full Course #46</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/b2HSqC0RGsM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/fyAW0W526RM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Introduction to Multithreading in Java | Process vs Thread | Java Full Course #47</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Thread Creation &amp; Lifecycle Explained from Scratch | Java Full Course #48</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/cVRdeQFP5IM</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1788,39 +1820,55 @@
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
     </row>
-    <row r="50" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B50" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C50" s="13"/>
-      <c r="D50" s="5"/>
+      <c r="C50" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>164</v>
+      </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B51" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="C51" s="13"/>
-      <c r="D51" s="5"/>
+      <c r="C51" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>166</v>
+      </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
     </row>
-    <row r="52" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B52" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="C52" s="13"/>
-      <c r="D52" s="5"/>
+      <c r="C52" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>167</v>
+      </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
     </row>
-    <row r="53" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B53" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C53" s="13"/>
-      <c r="D53" s="5"/>
+      <c r="C53" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>170</v>
+      </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
     </row>
@@ -2016,6 +2064,10 @@
     <hyperlink ref="D47" r:id="rId39" xr:uid="{9E9CFD17-8B4E-4159-A428-447A65AE33B9}"/>
     <hyperlink ref="D48" r:id="rId40" xr:uid="{EEFC57CB-B74A-4C45-8650-090249CDC424}"/>
     <hyperlink ref="D49" r:id="rId41" xr:uid="{E4D9CAFF-0AF5-4837-B77F-00BD2850517C}"/>
+    <hyperlink ref="D50" r:id="rId42" xr:uid="{ED2346CA-59B5-479D-8BBA-A0C05F174AE2}"/>
+    <hyperlink ref="D51" r:id="rId43" xr:uid="{75CC2455-0D21-4C9C-8D83-771E16989D04}"/>
+    <hyperlink ref="D52" r:id="rId44" xr:uid="{F8F457B2-C23B-4B65-8641-85AA50A0CC44}"/>
+    <hyperlink ref="D53" r:id="rId45" xr:uid="{C5D9EFD0-D3D8-481A-A7EA-F58DE789D54D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
learn about threadproblem-racecodition,visibility problem and odering problem
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC946E34-9269-48D1-A717-45622408BF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EABDF4-5EE6-465A-98D4-0365CD4D386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="175">
   <si>
     <t>video</t>
   </si>
@@ -625,6 +625,22 @@
   </si>
   <si>
     <t>https://youtu.be/cVRdeQFP5IM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Thread Methods | sleep, join, yield, interrupt, isAlive, priority &amp; more | Java Full Course #49</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/ZPxJby0GeOQ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Problems in Multithreading | Race Condition, Visibility, Ordering Explained | Java Full Course #50</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/lrrdN_c0HQ4</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1872,21 +1888,29 @@
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
     </row>
-    <row r="54" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B54" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="5"/>
+      <c r="C54" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>172</v>
+      </c>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
     </row>
-    <row r="55" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B55" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="5"/>
+      <c r="C55" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>174</v>
+      </c>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
     </row>
@@ -2068,6 +2092,8 @@
     <hyperlink ref="D51" r:id="rId43" xr:uid="{75CC2455-0D21-4C9C-8D83-771E16989D04}"/>
     <hyperlink ref="D52" r:id="rId44" xr:uid="{F8F457B2-C23B-4B65-8641-85AA50A0CC44}"/>
     <hyperlink ref="D53" r:id="rId45" xr:uid="{C5D9EFD0-D3D8-481A-A7EA-F58DE789D54D}"/>
+    <hyperlink ref="D54" r:id="rId46" xr:uid="{D691C1F5-E537-4203-946A-0CC0416B1063}"/>
+    <hyperlink ref="D55" r:id="rId47" xr:uid="{E6C2056C-D997-4EC0-988D-D0EF217C091E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
threadlocks list Java Locks | ReentrantLock, ReadWriteLock, StampedLock, Semaphore &
</commit_message>
<xml_diff>
--- a/Class-Updates-Tracker-Java.xlsx
+++ b/Class-Updates-Tracker-Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java utube\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EABDF4-5EE6-465A-98D4-0365CD4D386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3608DC68-C03B-47B8-86A6-417F477D4597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="187">
   <si>
     <t>video</t>
   </si>
@@ -202,445 +202,496 @@
     <t>Day17</t>
   </si>
   <si>
+    <t>oops piller2- polymorphism ,run time polymorphism(method overriding), compile time polymorphism(method overloading)</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>extra</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>how java programming language introduce ,why java compile and intreprate language and jvm jre and jdk</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/LBqE4YOvhyc</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/pdS8_smlsXA</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-VOO76LOCv4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>oops piller3-encapsulation ,packages and why make getters and setters  to access data</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-L9BcU6Xk2c</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day18</t>
+  </si>
+  <si>
+    <t>Day19</t>
+  </si>
+  <si>
+    <t>Day20</t>
+  </si>
+  <si>
+    <t>Day21</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> repeate&gt;&gt;oops pillers4 abstraction and piller 1 polymorphism repeate</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>repeate&gt;&gt;encapsulation and inheritance (piller3 and piller2)</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>oops piller4-abstraction and interface</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/jfLpzL1VW7Q</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/dDw99mE6EbQ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day22</t>
+  </si>
+  <si>
+    <t>Day23</t>
+  </si>
+  <si>
+    <t>Day24</t>
+  </si>
+  <si>
+    <t>interface deep dive,default method,functionl and marker interface</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/YLLFHuStkW8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/crVwHNW-fX8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">AutoBoxing, Abstract classes &amp; POJOs | Why only one public class in java file </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/0LaBK28_470</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Nested Classes type| 1)Static Nested, 2)Inner, 3)Local &amp;4)Anonymous Classes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">learn Immutable Classes in Java | How to Create Immutable Objects </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/vgQVz5OdFws</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/541Zpv6sOKo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day25</t>
+  </si>
+  <si>
+    <t>Day26</t>
+  </si>
+  <si>
+    <t>Day27</t>
+  </si>
+  <si>
+    <t>Day28</t>
+  </si>
+  <si>
+    <t>Day29</t>
+  </si>
+  <si>
+    <t>Day30</t>
+  </si>
+  <si>
+    <t>Day31</t>
+  </si>
+  <si>
+    <t>Day32</t>
+  </si>
+  <si>
+    <t>learn Object Class (equals, hashCode, toString)  which is most important in java</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java Enums | Why Not Use int/String for Constants? </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/oXhy5dT-0Qs</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/yfMWLZGEPwo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java I/O Deep Dive | InputStreams, System.in, Scanner vs BufferedReader</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Strings | String Pool, Immutability, Internals</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/N0b8lRXtK_Y</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/JcAD9a22Rks</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Strings Part 2 | All String Methods + StringBuilder vs StringBuffer</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Y7X_ReDF3x8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java Generics Deep Dive | Bounded Types using extends </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Wildcards in Generics |  extends, ? super | Java Full Course #28</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Opb2q2WSyes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/mW2OO6d6_BE</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">theory only-Java Collection Framework Explained | Data Structures + Complete Hierarchy </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/LVwpxEZ6uMQ</t>
+  </si>
+  <si>
+    <t>Iterable Interface in Java | Why Iterator Exists?</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Collection Interface Deep Dive | Methods &amp; Internals | Java Full Course #31</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/cazzzwdLAkQ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/OfNtIOGDqzY</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java List Interface Deep Dive | ArrayList, LinkedList, Vector, Stack </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day33</t>
+  </si>
+  <si>
+    <t>Day34</t>
+  </si>
+  <si>
+    <t>Day35</t>
+  </si>
+  <si>
+    <t>Day36</t>
+  </si>
+  <si>
+    <t>Day37</t>
+  </si>
+  <si>
+    <t>Day38</t>
+  </si>
+  <si>
+    <t>Day39</t>
+  </si>
+  <si>
+    <t>Day40</t>
+  </si>
+  <si>
+    <t>Day41</t>
+  </si>
+  <si>
+    <t>Day42</t>
+  </si>
+  <si>
+    <t>https://youtu.be/kzZ1TlGTWmY</t>
+  </si>
+  <si>
+    <t>Set &amp; Map Interface in Java | Internal Working of HashMap, HashSet &amp; TreeMap</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Set &amp; Map Methods Explained | EnumMaps, IdentityHashMaps &amp; More in collection framework</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/b1Uj_2MPBwA</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/zj0-JIc5oPw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Queue Interface Deep Dive | PriorityQueue &amp; Heap Explained | Java Full Course #35</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day43</t>
+  </si>
+  <si>
+    <t>Day44</t>
+  </si>
+  <si>
+    <t>Day45</t>
+  </si>
+  <si>
+    <t>Day46</t>
+  </si>
+  <si>
+    <t>Day47</t>
+  </si>
+  <si>
+    <t>Day48</t>
+  </si>
+  <si>
+    <t>Day49</t>
+  </si>
+  <si>
+    <t>https://youtu.be/uUo7AV02vJM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Comparable Interface in Java | Collections class | Comparing Objects | Java Full Course #36</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Lambdas &amp; Functional Interfaces | Comparator Interface | Java Full Course #37</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/0V-w2BywAM0</t>
+  </si>
+  <si>
+    <t>Lambdas &amp; Functional Interface Deep Dive | Method References &amp; Composition | Java Full Course #38</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/IsC0Ms2iFi8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/-jHyDEXHr_U</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Java Streams | Creation &amp; Architecture </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Day50</t>
+  </si>
+  <si>
+    <t>Day51</t>
+  </si>
+  <si>
+    <t>Day52</t>
+  </si>
+  <si>
+    <t>Day53</t>
+  </si>
+  <si>
+    <t>Day54</t>
+  </si>
+  <si>
+    <t>Day55</t>
+  </si>
+  <si>
+    <t>Day56</t>
+  </si>
+  <si>
+    <t>Day57</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xqfOH5EA8xo</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Java Stream Methods Deep Dive | All Intermediate &amp; Terminal Operations </t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/Q75kCaNa35Y</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Optional Explained from Scratch | All Methods + Streams Integration</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Parallel Streams in Java Explained | Primitive Optional Classes</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/zrtVQ1ev_0w</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Exception Handling from Scratch | Exceptions vs Errors |</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/mJg9iQZJEpw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Exception Hierarchy Deep Dive | throw vs throws | Custom Exceptions | Java Full Course #44</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/xTxscoajikw</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Memory Management Explained in Depth | Stack, Heap, Method Area &amp; PC | Java Full Course #45</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/kjETbH63Pco</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Heap Memory Deep Dive | Garbage Collection Algorithms Explained | Java Full Course #46</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/b2HSqC0RGsM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/fyAW0W526RM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Introduction to Multithreading in Java | Process vs Thread | Java Full Course #47</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Thread Creation &amp; Lifecycle Explained from Scratch | Java Full Course #48</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/cVRdeQFP5IM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Thread Methods | sleep, join, yield, interrupt, isAlive, priority &amp; more | Java Full Course #49</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/ZPxJby0GeOQ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Problems in Multithreading | Race Condition, Visibility, Ordering Explained | Java Full Course #50</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/lrrdN_c0HQ4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Monitor Locks in Java | Synchronized Keyword, Static Sync &amp; Custom Locks | Java Full Course #51</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/k9sURAu0xT8</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
     <t>https://youtu.be/GsqLYUAYGO4</t>
-  </si>
-  <si>
-    <t>oops piller2- polymorphism ,run time polymorphism(method overriding), compile time polymorphism(method overloading)</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>extra</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>how java programming language introduce ,why java compile and intreprate language and jvm jre and jdk</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/LBqE4YOvhyc</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/pdS8_smlsXA</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/-VOO76LOCv4</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>oops piller3-encapsulation ,packages and why make getters and setters  to access data</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/-L9BcU6Xk2c</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day18</t>
-  </si>
-  <si>
-    <t>Day19</t>
-  </si>
-  <si>
-    <t>Day20</t>
-  </si>
-  <si>
-    <t>Day21</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> repeate&gt;&gt;oops pillers4 abstraction and piller 1 polymorphism repeate</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>repeate&gt;&gt;encapsulation and inheritance (piller3 and piller2)</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>oops piller4-abstraction and interface</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/jfLpzL1VW7Q</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/dDw99mE6EbQ</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day22</t>
-  </si>
-  <si>
-    <t>Day23</t>
-  </si>
-  <si>
-    <t>Day24</t>
-  </si>
-  <si>
-    <t>interface deep dive,default method,functionl and marker interface</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/YLLFHuStkW8</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/crVwHNW-fX8</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">AutoBoxing, Abstract classes &amp; POJOs | Why only one public class in java file </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/0LaBK28_470</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Nested Classes type| 1)Static Nested, 2)Inner, 3)Local &amp;4)Anonymous Classes</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">learn Immutable Classes in Java | How to Create Immutable Objects </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/vgQVz5OdFws</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/541Zpv6sOKo</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day25</t>
-  </si>
-  <si>
-    <t>Day26</t>
-  </si>
-  <si>
-    <t>Day27</t>
-  </si>
-  <si>
-    <t>Day28</t>
-  </si>
-  <si>
-    <t>Day29</t>
-  </si>
-  <si>
-    <t>Day30</t>
-  </si>
-  <si>
-    <t>Day31</t>
-  </si>
-  <si>
-    <t>Day32</t>
-  </si>
-  <si>
-    <t>learn Object Class (equals, hashCode, toString)  which is most important in java</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Java Enums | Why Not Use int/String for Constants? </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/oXhy5dT-0Qs</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/yfMWLZGEPwo</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java I/O Deep Dive | InputStreams, System.in, Scanner vs BufferedReader</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Strings | String Pool, Immutability, Internals</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/N0b8lRXtK_Y</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/JcAD9a22Rks</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Strings Part 2 | All String Methods + StringBuilder vs StringBuffer</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/Y7X_ReDF3x8</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Java Generics Deep Dive | Bounded Types using extends </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Wildcards in Generics |  extends, ? super | Java Full Course #28</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/Opb2q2WSyes</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/mW2OO6d6_BE</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">theory only-Java Collection Framework Explained | Data Structures + Complete Hierarchy </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/LVwpxEZ6uMQ</t>
-  </si>
-  <si>
-    <t>Iterable Interface in Java | Why Iterator Exists?</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Collection Interface Deep Dive | Methods &amp; Internals | Java Full Course #31</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/cazzzwdLAkQ</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/OfNtIOGDqzY</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Java List Interface Deep Dive | ArrayList, LinkedList, Vector, Stack </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day33</t>
-  </si>
-  <si>
-    <t>Day34</t>
-  </si>
-  <si>
-    <t>Day35</t>
-  </si>
-  <si>
-    <t>Day36</t>
-  </si>
-  <si>
-    <t>Day37</t>
-  </si>
-  <si>
-    <t>Day38</t>
-  </si>
-  <si>
-    <t>Day39</t>
-  </si>
-  <si>
-    <t>Day40</t>
-  </si>
-  <si>
-    <t>Day41</t>
-  </si>
-  <si>
-    <t>Day42</t>
-  </si>
-  <si>
-    <t>https://youtu.be/kzZ1TlGTWmY</t>
-  </si>
-  <si>
-    <t>Set &amp; Map Interface in Java | Internal Working of HashMap, HashSet &amp; TreeMap</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Set &amp; Map Methods Explained | EnumMaps, IdentityHashMaps &amp; More in collection framework</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/b1Uj_2MPBwA</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/zj0-JIc5oPw</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Queue Interface Deep Dive | PriorityQueue &amp; Heap Explained | Java Full Course #35</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day43</t>
-  </si>
-  <si>
-    <t>Day44</t>
-  </si>
-  <si>
-    <t>Day45</t>
-  </si>
-  <si>
-    <t>Day46</t>
-  </si>
-  <si>
-    <t>Day47</t>
-  </si>
-  <si>
-    <t>Day48</t>
-  </si>
-  <si>
-    <t>Day49</t>
-  </si>
-  <si>
-    <t>https://youtu.be/uUo7AV02vJM</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Comparable Interface in Java | Collections class | Comparing Objects | Java Full Course #36</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Lambdas &amp; Functional Interfaces | Comparator Interface | Java Full Course #37</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/0V-w2BywAM0</t>
-  </si>
-  <si>
-    <t>Lambdas &amp; Functional Interface Deep Dive | Method References &amp; Composition | Java Full Course #38</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/IsC0Ms2iFi8</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/-jHyDEXHr_U</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduction to Java Streams | Creation &amp; Architecture </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Day50</t>
-  </si>
-  <si>
-    <t>Day51</t>
-  </si>
-  <si>
-    <t>Day52</t>
-  </si>
-  <si>
-    <t>Day53</t>
-  </si>
-  <si>
-    <t>Day54</t>
-  </si>
-  <si>
-    <t>Day55</t>
-  </si>
-  <si>
-    <t>Day56</t>
-  </si>
-  <si>
-    <t>Day57</t>
-  </si>
-  <si>
-    <t>Day58</t>
-  </si>
-  <si>
-    <t>Day59</t>
-  </si>
-  <si>
-    <t>https://youtu.be/xqfOH5EA8xo</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Java Stream Methods Deep Dive | All Intermediate &amp; Terminal Operations </t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/Q75kCaNa35Y</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Optional Explained from Scratch | All Methods + Streams Integration</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Parallel Streams in Java Explained | Primitive Optional Classes</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/zrtVQ1ev_0w</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Exception Handling from Scratch | Exceptions vs Errors |</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/mJg9iQZJEpw</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Exception Hierarchy Deep Dive | throw vs throws | Custom Exceptions | Java Full Course #44</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/xTxscoajikw</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Memory Management Explained in Depth | Stack, Heap, Method Area &amp; PC | Java Full Course #45</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/kjETbH63Pco</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Heap Memory Deep Dive | Garbage Collection Algorithms Explained | Java Full Course #46</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/b2HSqC0RGsM</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/fyAW0W526RM</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Introduction to Multithreading in Java | Process vs Thread | Java Full Course #47</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Java Thread Creation &amp; Lifecycle Explained from Scratch | Java Full Course #48</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/cVRdeQFP5IM</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Thread Methods | sleep, join, yield, interrupt, isAlive, priority &amp; more | Java Full Course #49</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/ZPxJby0GeOQ</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>Problems in Multithreading | Race Condition, Visibility, Ordering Explained | Java Full Course #50</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>https://youtu.be/lrrdN_c0HQ4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Inter Thread Communication in Java | wait(), notify(), notifyAll() Deep Dive | Java Full Course #52</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/EZS19NLnsvc</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Java Locks | ReentrantLock, ReadWriteLock, StampedLock, Semaphore &amp; Condition | #53</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/JW6-TCU0iS4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Lock-Free Concurrency in Java | AtomicVariables &amp; CAS Explained | Java Full Course #54</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/ujF2gNsCfBE</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Lock-Free Concurrency in Java - 2 | CAS Retry, Compare-and-Swap &amp; ABA Problem | #55</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/2nBJPpERul4</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>Executor Framework Deep Dive | ThreadPool, Future &amp; Callable | Java Full Course #56</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/VPtaTUSaBOM</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>CompletableFuture, Fork-Join Pool, ThreadLocal &amp; Virtual Threads | Java Full Course #57</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>https://youtu.be/FGN225TiXaE</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1193,7 +1244,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:F111"/>
+  <dimension ref="B1:F115"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
@@ -1254,13 +1305,13 @@
     </row>
     <row r="6" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -1291,7 +1342,7 @@
         <v>15</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F8" s="4"/>
     </row>
@@ -1420,15 +1471,15 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B18" s="14" t="s">
         <v>48</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="5" t="s">
         <v>53</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>174</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -1438,10 +1489,10 @@
         <v>49</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -1451,10 +1502,10 @@
         <v>50</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -1464,10 +1515,10 @@
         <v>51</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -1477,509 +1528,537 @@
         <v>52</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
     <row r="23" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B23" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C23" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B24" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
     <row r="25" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B25" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B26" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C26" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
     <row r="27" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B27" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
     <row r="28" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B28" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C28" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
     <row r="29" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B29" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
     <row r="30" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B30" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C30" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
     <row r="31" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B31" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
     <row r="32" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B32" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B33" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C33" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>102</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>103</v>
       </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
     <row r="34" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B34" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
     <row r="35" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B35" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
     <row r="36" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B36" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C36" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>108</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>109</v>
       </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
     </row>
     <row r="37" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B37" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B38" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
     <row r="39" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B39" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C39" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>125</v>
       </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B40" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
     </row>
     <row r="41" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B41" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B42" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="D42" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>138</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
     </row>
     <row r="43" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B43" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C43" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D43" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
     </row>
     <row r="44" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B44" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
     <row r="45" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B45" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
     </row>
     <row r="46" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B46" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
     </row>
     <row r="47" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B47" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B48" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
     </row>
     <row r="49" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B49" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
     </row>
     <row r="50" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B50" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
     </row>
     <row r="51" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B51" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
     </row>
     <row r="52" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B52" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
     </row>
     <row r="53" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B53" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
     </row>
     <row r="54" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B54" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
     </row>
     <row r="55" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B55" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
     </row>
-    <row r="56" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B56" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C56" s="13"/>
-      <c r="D56" s="5"/>
+        <v>143</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>173</v>
+      </c>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
     </row>
-    <row r="57" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B57" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C57" s="13"/>
-      <c r="D57" s="5"/>
+        <v>144</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>176</v>
+      </c>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
     </row>
-    <row r="58" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B58" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="C58" s="13"/>
-      <c r="D58" s="5"/>
+        <v>145</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>178</v>
+      </c>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
     </row>
-    <row r="59" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B59" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="C59" s="13"/>
-      <c r="D59" s="5"/>
+        <v>146</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>180</v>
+      </c>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B60" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>182</v>
+      </c>
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
     </row>
-    <row r="61" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B61" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="C61" s="13"/>
-      <c r="D61" s="5"/>
+        <v>148</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>184</v>
+      </c>
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
     </row>
-    <row r="62" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B62" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="C62" s="13"/>
-      <c r="D62" s="5"/>
+        <v>149</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>186</v>
+      </c>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
     </row>
     <row r="63" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B63" s="14" t="s">
-        <v>151</v>
+        <v>54</v>
       </c>
       <c r="C63" s="13"/>
       <c r="D63" s="5"/>
@@ -1988,29 +2067,61 @@
     </row>
     <row r="64" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B64" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="C64" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="C64" s="13"/>
       <c r="D64" s="5"/>
       <c r="E64" s="4"/>
       <c r="F64" s="4"/>
     </row>
-    <row r="65" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B65" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C65" s="13"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+    </row>
+    <row r="66" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B66" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C66" s="13"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+    </row>
+    <row r="67" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B67" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" s="13"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+    </row>
+    <row r="68" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B68" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+    </row>
+    <row r="69" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="71" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="81" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="82" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="83" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2025,25 +2136,29 @@
     <row r="92" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="93" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="94" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="96" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="97" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="98" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" spans="2:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="100" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="101" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B102" s="6"/>
-    </row>
+    <row r="102" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="103" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="105" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="106" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B106" s="6"/>
+    </row>
     <row r="107" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="108" spans="2:2" ht="15.65" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="109" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="110" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" spans="2:2" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="111" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="112" spans="2:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="113" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="114" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="115" ht="28.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="5"/>
   <hyperlinks>
@@ -2094,6 +2209,14 @@
     <hyperlink ref="D53" r:id="rId45" xr:uid="{C5D9EFD0-D3D8-481A-A7EA-F58DE789D54D}"/>
     <hyperlink ref="D54" r:id="rId46" xr:uid="{D691C1F5-E537-4203-946A-0CC0416B1063}"/>
     <hyperlink ref="D55" r:id="rId47" xr:uid="{E6C2056C-D997-4EC0-988D-D0EF217C091E}"/>
+    <hyperlink ref="D56" r:id="rId48" xr:uid="{32805016-E539-4C67-9A2A-0857672F8906}"/>
+    <hyperlink ref="D18" r:id="rId49" xr:uid="{3D0E2D80-E679-4679-854E-B8A3F099FC43}"/>
+    <hyperlink ref="D57" r:id="rId50" xr:uid="{E6883963-E74E-419A-8DF9-55E302F3E65D}"/>
+    <hyperlink ref="D58" r:id="rId51" xr:uid="{50AD8637-9C5E-44EC-9648-1B393C8CCE8B}"/>
+    <hyperlink ref="D59" r:id="rId52" xr:uid="{9B223346-2F5F-4C33-A010-5A7B29F160AF}"/>
+    <hyperlink ref="D60" r:id="rId53" xr:uid="{D95EBACB-70F7-401C-B41E-F8E40797788F}"/>
+    <hyperlink ref="D61" r:id="rId54" xr:uid="{9506C596-41F8-4F45-BDE0-8FC806698A23}"/>
+    <hyperlink ref="D62" r:id="rId55" xr:uid="{76A978A3-87BB-4D66-BEC2-5726F855AA0A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>